<commit_message>
update the chip 8 project
</commit_message>
<xml_diff>
--- a/server/projects/sheet-8.xlsx
+++ b/server/projects/sheet-8.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="42">
   <si>
     <t>Power</t>
   </si>
@@ -117,10 +117,28 @@
     <t>01</t>
   </si>
   <si>
+    <t>61</t>
+  </si>
+  <si>
+    <t>02</t>
+  </si>
+  <si>
+    <t>62</t>
+  </si>
+  <si>
+    <t>03</t>
+  </si>
+  <si>
+    <t>71</t>
+  </si>
+  <si>
+    <t>72</t>
+  </si>
+  <si>
     <t>12</t>
   </si>
   <si>
-    <t>02</t>
+    <t>06</t>
   </si>
 </sst>
 </file>
@@ -215,7 +233,7 @@
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment vertical="bottom"/>
+      <alignment readingOrder="0" vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
@@ -228,7 +246,7 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="49" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="2" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" vertical="bottom"/>
+      <alignment vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment vertical="bottom"/>
@@ -520,7 +538,7 @@
       <c r="Z1" s="5"/>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="6" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="b">
@@ -552,7 +570,7 @@
       <c r="Z2" s="5"/>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="7"/>
@@ -582,7 +600,7 @@
       <c r="Z3" s="5"/>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="6" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="7" t="str">
@@ -626,7 +644,7 @@
       <c r="Z4" s="5"/>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="6" t="s">
         <v>4</v>
       </c>
       <c r="B5" s="9" t="str">
@@ -634,21 +652,21 @@
         <v>0</v>
       </c>
       <c r="C5" s="9"/>
-      <c r="D5" s="9">
-        <f>IF(C39 = "A", H39, D5)</f>
-        <v>0</v>
+      <c r="D5" s="9" t="str">
+        <f>IF(C4 = "A", G4, D5)</f>
+        <v>#REF!</v>
       </c>
       <c r="E5" s="10" t="str">
-        <f>IFS(C4 = "6", IF(D4 = "0", G4, E5),C4 = "7", IF(D4="0", DEC2HEX(MOD(HEX2DEC(E5)+HEX2DEC(G4), 256)), E5), TRUE, E5)</f>
+        <f>IFS(C4 = "6", IF(D4 = "0", VALUE(G4), E5),C4 = "7", IF(D4="0", DEC2HEX(MOD(HEX2DEC(E5)+HEX2DEC(G4), 256)), E5), TRUE, E5)</f>
         <v>#REF!</v>
       </c>
-      <c r="F5" s="11">
-        <f>IFS(C39 = "6", IF(D39 = "1", G39, F5),  C39="7", IF(D39="1", DEC2HEX(MOD(HEX2DEC(F5)+HEX2DEC(G39), 256)), F5), TRUE, F5)</f>
-        <v>0</v>
+      <c r="F5" s="11" t="str">
+        <f>IFS(C4 = "6", IF(D4 = "1", VALUE(G4), F5),C4 = "7", IF(D4="1", DEC2HEX(MOD(HEX2DEC(F5)+HEX2DEC(G4), 256)), F5), TRUE, F5)</f>
+        <v>#REF!</v>
       </c>
-      <c r="G5" s="11">
-        <f>IFS(C39 = "6", IF(D39 = "2", G39, G5), C39="7", IF(D39="2", DEC2HEX(MOD(HEX2DEC(G5)+HEX2DEC(G39), 256)), G5), TRUE, G5)</f>
-        <v>0</v>
+      <c r="G5" s="11" t="str">
+        <f>IFS(C4 = "6", IF(D4 = "2", VALUE(G4), G5),C4 = "7", IF(D4="2", DEC2HEX(MOD(HEX2DEC(G5)+HEX2DEC(G4), 256)), G5), TRUE, G5)</f>
+        <v>#REF!</v>
       </c>
       <c r="H5" s="11">
         <f>IFS(C39 = "6", IF(D39 = "3", G39, H5),  C39="7", IF(D39="3", DEC2HEX(MOD(HEX2DEC(H5)+HEX2DEC(G39), 256)), H5),TRUE, H5)</f>
@@ -710,7 +728,7 @@
       <c r="Z5" s="5"/>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B6" s="12"/>
@@ -30924,59 +30942,75 @@
       <c r="B513" s="19"/>
     </row>
     <row r="514">
-      <c r="A514" s="21" t="s">
+      <c r="A514" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="B514" s="19"/>
+    </row>
+    <row r="515">
+      <c r="A515" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="B515" s="19"/>
+    </row>
+    <row r="516">
+      <c r="A516" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="B516" s="19"/>
+    </row>
+    <row r="517">
+      <c r="A517" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="B517" s="19"/>
+    </row>
+    <row r="518">
+      <c r="A518" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="B514" s="19"/>
-    </row>
-    <row r="515">
-      <c r="A515" s="21" t="s">
+      <c r="B518" s="19"/>
+    </row>
+    <row r="519">
+      <c r="A519" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="B515" s="19"/>
-    </row>
-    <row r="516">
-      <c r="A516" s="22" t="s">
-        <v>34</v>
+      <c r="B519" s="19"/>
+    </row>
+    <row r="520">
+      <c r="A520" s="22" t="s">
+        <v>38</v>
       </c>
-      <c r="B516" s="19"/>
-    </row>
-    <row r="517">
-      <c r="A517" s="22" t="s">
-        <v>35</v>
+      <c r="B520" s="19"/>
+    </row>
+    <row r="521">
+      <c r="A521" s="22" t="s">
+        <v>33</v>
       </c>
-      <c r="B517" s="19"/>
-    </row>
-    <row r="518">
-      <c r="A518" s="21"/>
-      <c r="B518" s="19"/>
-    </row>
-    <row r="519">
-      <c r="A519" s="22"/>
-      <c r="B519" s="19"/>
-    </row>
-    <row r="520">
-      <c r="A520" s="21"/>
-      <c r="B520" s="19"/>
-    </row>
-    <row r="521">
-      <c r="A521" s="21"/>
       <c r="B521" s="19"/>
     </row>
     <row r="522">
-      <c r="A522" s="21"/>
+      <c r="A522" s="22" t="s">
+        <v>39</v>
+      </c>
       <c r="B522" s="19"/>
     </row>
     <row r="523">
-      <c r="A523" s="22"/>
+      <c r="A523" s="22" t="s">
+        <v>33</v>
+      </c>
       <c r="B523" s="19"/>
     </row>
     <row r="524">
-      <c r="A524" s="21"/>
+      <c r="A524" s="22" t="s">
+        <v>40</v>
+      </c>
       <c r="B524" s="19"/>
     </row>
     <row r="525">
-      <c r="A525" s="21"/>
+      <c r="A525" s="22" t="s">
+        <v>41</v>
+      </c>
       <c r="B525" s="19"/>
     </row>
     <row r="526">

</xml_diff>